<commit_message>
added new data for Policia de Puerto Rico
</commit_message>
<xml_diff>
--- a/data/Negociado_de_Policia/npprVDedad.xlsx
+++ b/data/Negociado_de_Policia/npprVDedad.xlsx
@@ -1,33 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\orlando.hernandez\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\Negociado_de_Policia\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21BCB29C-E4E5-4813-AF67-3FC340FB8519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12135" activeTab="3"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13056" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2021" sheetId="2" r:id="rId1"/>
     <sheet name="2022" sheetId="3" r:id="rId2"/>
     <sheet name="2023" sheetId="4" r:id="rId3"/>
     <sheet name="2024" sheetId="5" r:id="rId4"/>
+    <sheet name="2025" sheetId="6" r:id="rId5"/>
+    <sheet name="2026" sheetId="7" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="19">
   <si>
     <t>Desconocida</t>
   </si>
@@ -89,7 +103,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -134,7 +148,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -411,14 +425,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="41.7109375" customWidth="1"/>
+    <col min="1" max="1" width="41.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -435,11 +449,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>13</v>
       </c>
       <c r="B2">
+        <f>SUM(C2:E2)</f>
         <v>11</v>
       </c>
       <c r="C2">
@@ -452,11 +467,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
       <c r="B3">
+        <f t="shared" ref="B3:B15" si="0">SUM(C3:E3)</f>
         <v>44</v>
       </c>
       <c r="C3">
@@ -469,11 +485,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
       <c r="B4">
+        <f t="shared" si="0"/>
         <v>194</v>
       </c>
       <c r="C4">
@@ -486,11 +503,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
       <c r="B5">
+        <f t="shared" si="0"/>
         <v>1086</v>
       </c>
       <c r="C5">
@@ -503,11 +521,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
       <c r="B6">
+        <f t="shared" si="0"/>
         <v>1361</v>
       </c>
       <c r="C6">
@@ -520,11 +539,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
       <c r="B7">
+        <f t="shared" si="0"/>
         <v>1221</v>
       </c>
       <c r="C7">
@@ -537,11 +557,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
       <c r="B8">
+        <f t="shared" si="0"/>
         <v>942</v>
       </c>
       <c r="C8">
@@ -554,11 +575,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>6</v>
       </c>
       <c r="B9">
+        <f t="shared" si="0"/>
         <v>759</v>
       </c>
       <c r="C9">
@@ -571,11 +593,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>5</v>
       </c>
       <c r="B10">
+        <f t="shared" si="0"/>
         <v>514</v>
       </c>
       <c r="C10">
@@ -588,11 +611,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>4</v>
       </c>
       <c r="B11">
+        <f t="shared" si="0"/>
         <v>334</v>
       </c>
       <c r="C11">
@@ -605,11 +629,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>3</v>
       </c>
       <c r="B12">
+        <f t="shared" si="0"/>
         <v>217</v>
       </c>
       <c r="C12">
@@ -622,11 +647,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>2</v>
       </c>
       <c r="B13">
+        <f t="shared" si="0"/>
         <v>144</v>
       </c>
       <c r="C13">
@@ -639,11 +665,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>1</v>
       </c>
       <c r="B14">
+        <f t="shared" si="0"/>
         <v>169</v>
       </c>
       <c r="C14">
@@ -656,11 +683,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>0</v>
       </c>
       <c r="B15">
+        <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="C15">
@@ -679,18 +707,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="58.42578125" style="1" customWidth="1"/>
-    <col min="2" max="3" width="13.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="58.44140625" style="1" customWidth="1"/>
+    <col min="2" max="3" width="13.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
@@ -707,7 +735,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
@@ -721,11 +749,11 @@
         <v>0</v>
       </c>
       <c r="E2" s="1">
-        <f t="shared" ref="E2:E15" si="0">SUM(B2:D2)</f>
+        <f>SUM(B2:D2)</f>
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -739,11 +767,11 @@
         <v>0</v>
       </c>
       <c r="E3" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E3:E15" si="0">SUM(B3:D3)</f>
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -761,7 +789,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -779,7 +807,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
@@ -797,7 +825,7 @@
         <v>1135</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -815,7 +843,7 @@
         <v>1022</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -833,7 +861,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
@@ -851,7 +879,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
@@ -869,7 +897,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
@@ -887,7 +915,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>3</v>
       </c>
@@ -905,7 +933,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
@@ -923,7 +951,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>1</v>
       </c>
@@ -941,7 +969,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
@@ -965,18 +993,18 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="27.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="27.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="1"/>
+    <col min="4" max="4" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
@@ -993,246 +1021,246 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B2" s="1">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C2" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D2" s="1">
         <v>0</v>
       </c>
       <c r="E2" s="1">
-        <f t="shared" ref="E2:E15" si="0">SUM(B2:D2)</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <f>SUM(B2:D2)</f>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B3" s="1">
-        <v>16</v>
+        <v>57</v>
       </c>
       <c r="C3" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D3" s="1">
         <v>0</v>
       </c>
       <c r="E3" s="1">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" ref="E3:E15" si="0">SUM(B3:D3)</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="1">
-        <v>40</v>
+        <v>169</v>
       </c>
       <c r="C4" s="1">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="D4" s="1">
         <v>0</v>
       </c>
       <c r="E4" s="1">
         <f t="shared" si="0"/>
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="1">
-        <v>262</v>
+        <v>955</v>
       </c>
       <c r="C5" s="1">
-        <v>39</v>
+        <v>140</v>
       </c>
       <c r="D5" s="1">
         <v>0</v>
       </c>
       <c r="E5" s="1">
         <f t="shared" si="0"/>
-        <v>301</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1095</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="1">
-        <v>355</v>
+        <v>1179</v>
       </c>
       <c r="C6" s="1">
-        <v>62</v>
+        <v>218</v>
       </c>
       <c r="D6" s="1">
         <v>0</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="0"/>
-        <v>417</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1397</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="1">
-        <v>299</v>
+        <v>1099</v>
       </c>
       <c r="C7" s="1">
-        <v>65</v>
+        <v>205</v>
       </c>
       <c r="D7" s="1">
         <v>0</v>
       </c>
       <c r="E7" s="1">
         <f t="shared" si="0"/>
-        <v>364</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1304</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="1">
-        <v>186</v>
+        <v>866</v>
       </c>
       <c r="C8" s="1">
-        <v>49</v>
+        <v>208</v>
       </c>
       <c r="D8" s="1">
         <v>0</v>
       </c>
       <c r="E8" s="1">
         <f t="shared" si="0"/>
-        <v>235</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B9" s="1">
-        <v>226</v>
+        <v>680</v>
       </c>
       <c r="C9" s="1">
-        <v>31</v>
+        <v>168</v>
       </c>
       <c r="D9" s="1">
         <v>0</v>
       </c>
       <c r="E9" s="1">
         <f t="shared" si="0"/>
-        <v>257</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B10" s="1">
-        <v>366</v>
+        <v>519</v>
       </c>
       <c r="C10" s="1">
-        <v>37</v>
+        <v>127</v>
       </c>
       <c r="D10" s="1">
         <v>0</v>
       </c>
       <c r="E10" s="1">
         <f t="shared" si="0"/>
-        <v>403</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B11" s="1">
-        <v>84</v>
+        <v>311</v>
       </c>
       <c r="C11" s="1">
-        <v>28</v>
+        <v>88</v>
       </c>
       <c r="D11" s="1">
         <v>0</v>
       </c>
       <c r="E11" s="1">
         <f t="shared" si="0"/>
-        <v>112</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B12" s="1">
-        <v>60</v>
+        <v>189</v>
       </c>
       <c r="C12" s="1">
-        <v>14</v>
+        <v>73</v>
       </c>
       <c r="D12" s="1">
         <v>0</v>
       </c>
       <c r="E12" s="1">
         <f t="shared" si="0"/>
-        <v>74</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B13" s="1">
-        <v>28</v>
+        <v>109</v>
       </c>
       <c r="C13" s="1">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="D13" s="1">
         <v>0</v>
       </c>
       <c r="E13" s="1">
         <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B14" s="1">
-        <v>51</v>
+        <v>168</v>
       </c>
       <c r="C14" s="1">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="D14" s="1">
         <v>0</v>
       </c>
       <c r="E14" s="1">
         <f t="shared" si="0"/>
-        <v>72</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B15" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" s="1">
         <v>0</v>
@@ -1242,7 +1270,7 @@
       </c>
       <c r="E15" s="1">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1251,18 +1279,18 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="27.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="15.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="27.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
@@ -1279,48 +1307,50 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B2" s="1">
-        <v>18</v>
+        <f>2+17</f>
+        <v>19</v>
       </c>
       <c r="C2" s="1">
+        <f>0+0</f>
         <v>0</v>
       </c>
       <c r="D2" s="1">
         <v>0</v>
       </c>
       <c r="E2" s="1">
-        <f>SUM(B2:D2)</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" ref="E2:E15" si="0">SUM(B2:D2)</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B3" s="1">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C3" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D3" s="1">
         <v>0</v>
       </c>
       <c r="E3" s="1">
-        <f>SUM(B3:D3)</f>
-        <v>59</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="1">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="C4" s="1">
         <v>18</v>
@@ -1329,191 +1359,765 @@
         <v>0</v>
       </c>
       <c r="E4" s="1">
-        <f>SUM(B4:D4)</f>
-        <v>187</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="1">
-        <v>1039</v>
+        <v>1101</v>
       </c>
       <c r="C5" s="1">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="D5" s="1">
         <v>0</v>
       </c>
       <c r="E5" s="1">
-        <f>SUM(B5:D5)</f>
-        <v>1202</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>1272</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="1">
-        <v>1390</v>
+        <v>1499</v>
       </c>
       <c r="C6" s="1">
-        <v>257</v>
+        <v>279</v>
       </c>
       <c r="D6" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E6" s="1">
-        <f>SUM(B6:D6)</f>
-        <v>1649</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>1778</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="1">
+        <v>1366</v>
+      </c>
+      <c r="C7" s="1">
+        <v>268</v>
+      </c>
+      <c r="D7" s="1">
+        <v>1</v>
+      </c>
+      <c r="E7" s="1">
+        <f t="shared" si="0"/>
+        <v>1635</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1">
+        <v>1062</v>
+      </c>
+      <c r="C8" s="1">
+        <v>272</v>
+      </c>
+      <c r="D8" s="1">
+        <v>2</v>
+      </c>
+      <c r="E8" s="1">
+        <f t="shared" si="0"/>
+        <v>1336</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="1">
+        <v>862</v>
+      </c>
+      <c r="C9" s="1">
+        <v>174</v>
+      </c>
+      <c r="D9" s="1">
+        <v>1</v>
+      </c>
+      <c r="E9" s="1">
+        <f t="shared" si="0"/>
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="1">
+        <v>602</v>
+      </c>
+      <c r="C10" s="1">
+        <v>168</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0</v>
+      </c>
+      <c r="E10" s="1">
+        <f t="shared" si="0"/>
+        <v>770</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="1">
+        <v>418</v>
+      </c>
+      <c r="C11" s="1">
+        <v>99</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0</v>
+      </c>
+      <c r="E11" s="1">
+        <f t="shared" si="0"/>
+        <v>517</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="1">
+        <v>274</v>
+      </c>
+      <c r="C12" s="1">
+        <v>89</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0</v>
+      </c>
+      <c r="E12" s="1">
+        <f t="shared" si="0"/>
+        <v>363</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B13" s="1">
+        <v>180</v>
+      </c>
+      <c r="C13" s="1">
+        <v>62</v>
+      </c>
+      <c r="D13" s="1">
+        <v>0</v>
+      </c>
+      <c r="E13" s="1">
+        <f t="shared" si="0"/>
+        <v>242</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="1">
+        <v>204</v>
+      </c>
+      <c r="C14" s="1">
+        <v>83</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1">
+        <f t="shared" si="0"/>
+        <v>287</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B15" s="1">
+        <v>1</v>
+      </c>
+      <c r="C15" s="1">
+        <v>0</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24FB097A-1CA8-4290-8FD4-94F2A1DA342E}">
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="27.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.109375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="1">
+        <f>3+14</f>
+        <v>17</v>
+      </c>
+      <c r="C2" s="1">
+        <f>0+1</f>
+        <v>1</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
+        <f t="shared" ref="E2:E15" si="0">SUM(B2:D2)</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1">
+        <v>50</v>
+      </c>
+      <c r="C3" s="1">
+        <v>12</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1">
+        <f t="shared" si="0"/>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="1">
+        <v>185</v>
+      </c>
+      <c r="C4" s="1">
+        <v>17</v>
+      </c>
+      <c r="D4" s="1">
+        <v>2</v>
+      </c>
+      <c r="E4" s="1">
+        <f t="shared" si="0"/>
+        <v>204</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="1">
+        <v>962</v>
+      </c>
+      <c r="C5" s="1">
+        <v>170</v>
+      </c>
+      <c r="D5" s="1">
+        <v>3</v>
+      </c>
+      <c r="E5" s="1">
+        <f t="shared" si="0"/>
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1">
         <v>1277</v>
       </c>
+      <c r="C6" s="1">
+        <v>239</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1">
+        <f t="shared" si="0"/>
+        <v>1517</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="1">
+        <v>1257</v>
+      </c>
       <c r="C7" s="1">
-        <v>246</v>
+        <v>271</v>
+      </c>
+      <c r="D7" s="1">
+        <v>1</v>
+      </c>
+      <c r="E7" s="1">
+        <f t="shared" si="0"/>
+        <v>1529</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1">
+        <v>980</v>
+      </c>
+      <c r="C8" s="1">
+        <v>239</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0</v>
+      </c>
+      <c r="E8" s="1">
+        <f t="shared" si="0"/>
+        <v>1219</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="1">
+        <v>758</v>
+      </c>
+      <c r="C9" s="1">
+        <v>178</v>
+      </c>
+      <c r="D9" s="1">
+        <v>3</v>
+      </c>
+      <c r="E9" s="1">
+        <f t="shared" si="0"/>
+        <v>939</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="1">
+        <v>566</v>
+      </c>
+      <c r="C10" s="1">
+        <v>156</v>
+      </c>
+      <c r="D10" s="1">
+        <v>1</v>
+      </c>
+      <c r="E10" s="1">
+        <f t="shared" si="0"/>
+        <v>723</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="1">
+        <v>369</v>
+      </c>
+      <c r="C11" s="1">
+        <v>112</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1</v>
+      </c>
+      <c r="E11" s="1">
+        <f t="shared" si="0"/>
+        <v>482</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="1">
+        <v>205</v>
+      </c>
+      <c r="C12" s="1">
+        <v>84</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0</v>
+      </c>
+      <c r="E12" s="1">
+        <f t="shared" si="0"/>
+        <v>289</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B13" s="1">
+        <v>134</v>
+      </c>
+      <c r="C13" s="1">
+        <v>60</v>
+      </c>
+      <c r="D13" s="1">
+        <v>1</v>
+      </c>
+      <c r="E13" s="1">
+        <f t="shared" si="0"/>
+        <v>195</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="1">
+        <v>198</v>
+      </c>
+      <c r="C14" s="1">
+        <v>84</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1">
+        <f t="shared" si="0"/>
+        <v>282</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B15" s="1">
+        <v>1</v>
+      </c>
+      <c r="C15" s="1">
+        <v>0</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{908DE649-C3E4-4870-A377-EDA19EBF3F40}">
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="27.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.109375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="1">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
+        <f t="shared" ref="E2:E15" si="0">SUM(B2:D2)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="1">
+        <v>48</v>
+      </c>
+      <c r="C4" s="1">
+        <v>11</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1">
+        <f t="shared" si="0"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="1">
+        <v>234</v>
+      </c>
+      <c r="C5" s="1">
+        <v>48</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1">
+        <f t="shared" si="0"/>
+        <v>282</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1">
+        <v>373</v>
+      </c>
+      <c r="C6" s="1">
+        <v>67</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1">
+        <f t="shared" si="0"/>
+        <v>441</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="1">
+        <v>347</v>
+      </c>
+      <c r="C7" s="1">
+        <v>67</v>
       </c>
       <c r="D7" s="1">
         <v>4</v>
       </c>
       <c r="E7" s="1">
-        <f>SUM(B7:D7)</f>
-        <v>1527</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>418</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="1">
-        <v>991</v>
+        <v>259</v>
       </c>
       <c r="C8" s="1">
-        <v>254</v>
+        <v>62</v>
       </c>
       <c r="D8" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="1">
-        <f>SUM(B8:D8)</f>
-        <v>1246</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>321</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B9" s="1">
-        <v>809</v>
+        <v>215</v>
       </c>
       <c r="C9" s="1">
-        <v>160</v>
+        <v>69</v>
       </c>
       <c r="D9" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9" s="1">
-        <f>SUM(B9:D9)</f>
-        <v>970</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>286</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B10" s="1">
-        <v>551</v>
+        <v>182</v>
       </c>
       <c r="C10" s="1">
-        <v>151</v>
+        <v>42</v>
       </c>
       <c r="D10" s="1">
         <v>0</v>
       </c>
       <c r="E10" s="1">
-        <f>SUM(B10:D10)</f>
-        <v>702</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>224</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B11" s="1">
-        <v>384</v>
+        <v>98</v>
       </c>
       <c r="C11" s="1">
-        <v>94</v>
+        <v>29</v>
       </c>
       <c r="D11" s="1">
         <v>1</v>
       </c>
       <c r="E11" s="1">
-        <f>SUM(B11:D11)</f>
-        <v>479</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B12" s="1">
-        <v>256</v>
+        <v>53</v>
       </c>
       <c r="C12" s="1">
-        <v>79</v>
+        <v>20</v>
       </c>
       <c r="D12" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E12" s="1">
-        <f>SUM(B12:D12)</f>
-        <v>335</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B13" s="1">
-        <v>172</v>
+        <v>28</v>
       </c>
       <c r="C13" s="1">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="D13" s="1">
         <v>0</v>
       </c>
       <c r="E13" s="1">
-        <f>SUM(B13:D13)</f>
-        <v>228</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B14" s="1">
-        <v>193</v>
+        <v>52</v>
       </c>
       <c r="C14" s="1">
-        <v>73</v>
+        <v>28</v>
       </c>
       <c r="D14" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="1">
-        <f>SUM(B14:D14)</f>
-        <v>266</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
@@ -1521,14 +2125,14 @@
         <v>1</v>
       </c>
       <c r="C15" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="1">
-        <f>SUM(B15:D15)</f>
-        <v>3</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>